<commit_message>
Update 3 posts with extended content (2026-09-21)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -56424,7 +56424,8 @@
 分泌されるホルモンも違う。  
 ポルノ＝ドーパミンのみ（空虚）  
 セ〇クス＝ドーパミン＋オキシトシン
-＋セロトニン（充足）</t>
+＋セロトニン（充足）  
+「女はコスパ悪い」とか抜かしてたら、一生埋まらないものを抱えながら生きる最悪な人生になるよ。</t>
         </is>
       </c>
       <c r="C1917" t="n">
@@ -56450,7 +56451,9 @@
           <t>スマホ中毒の本当の恐ろしさは、中毒がデフォルトになりすぎて誰も中毒だと気づかないところにある。
 電車、育児、歩行中、インフラ。
 あらゆる隙間にスマホが入ってきた。
-その状態で脱スマホ中毒を語ると「反テクノロジーですか？」「スピってますか？」でレッテルを貼られて終わる。</t>
+その状態で脱スマホ中毒を語ると「反テクノロジーですか？」「スピってますか？」でレッテルを貼られて終わる。
+実際に注意持続時間の低下、睡眠の質の悪化、幸福度低下等の実害は証明されており、宗教でも倫理でもない話をしているのに陰謀論者扱いされる。
+これにはディストピア的な恐怖を感じる。</t>
         </is>
       </c>
       <c r="C1918" t="n">
@@ -56481,7 +56484,8 @@
 ・「オナ禁してテストステロン爆上げ」 
 →筋トレもしろ  
 ・「自分を磨けば女性から来てくれる」
- →受け身が許されるのはTOP1％のみ</t>
+ →受け身が許されるのはTOP1％のみ  
+すべて俺が通ってきた道。</t>
         </is>
       </c>
       <c r="C1919" t="n">

</xml_diff>

<commit_message>
Add morning post 2026-10-08: 起床3秒
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -11,7 +11,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -50,9 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2133"/>
+  <dimension ref="A1:G2134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62802,6 +62805,26 @@
         </is>
       </c>
     </row>
+    <row r="2134">
+      <c r="A2134" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>堕落を治すには起床3秒が勝負。
+スマホに手を伸ばすか、
+歯ブラシに手を伸ばすか。
+「朝活をやろう」なんて考えなくていい。
+起床直後に歯ブラシに手を伸ばすことだけ意識すれば、
+あとは流れで上手くいきやすい。</t>
+        </is>
+      </c>
+      <c r="E2134" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-10-09: 大学モテ攻略
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2134"/>
+  <dimension ref="A1:G2135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62825,6 +62825,29 @@
         </is>
       </c>
     </row>
+    <row r="2135">
+      <c r="A2135" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>モテ攻略に大学はターニングポイントになる。
+・サークル、ゼミ、バイト
+・女側もオープン
+・童貞でも引け目がない
+・女も処女5~7割
+・失敗しても次のチャンスがある
+私は童貞チー牛時代に、
+講義後にナンパしたのが最初。
+私文は特にチャンスが多い。</t>
+        </is>
+      </c>
+      <c r="E2135" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix post 2026-10-10 19:00: add 快楽主義の末路
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -59117,14 +59117,16 @@
       </c>
       <c r="B2005" t="inlineStr">
         <is>
-          <t>甘い言葉に耳を傾けたら人生詰み。 
-・「嫌ならやめていい」 
-・「無理しなくていい」 
-・「若い内に遊ぶべき」 
-・「他人と比べなくていい」 
-・「好きなことだけで生きる」  
-これらの甘言を真に受けた 
-19歳の私は実家でニートしながら ゲーム、ポルノ、TikTokの毎日だった。</t>
+          <t>甘い言葉に耳を傾けたら人生詰み。
+・「嫌ならやめていい」
+・「無理しなくていい」
+・「若い内に遊ぶべき」
+・「他人と比べなくていい」
+・「好きなことだけで生きる」
+これらの甘言を真に受けた
+19歳の私は実家でニートしながら
+ゲーム、ポルノ、TikTokの毎日だった。
+快楽主義の末路はプライドだけ高いゴミ人間。</t>
         </is>
       </c>
       <c r="C2005" t="n">

</xml_diff>

<commit_message>
Add image to British guard post (row 2018)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -59543,6 +59543,11 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="G2018" t="inlineStr">
+        <is>
+          <t>images/british_guard.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="2019">
       <c r="A2019" t="inlineStr">

</xml_diff>

<commit_message>
Add bulking excuses post (row 2140)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2139"/>
+  <dimension ref="A1:G2140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62962,6 +62962,43 @@
         </is>
       </c>
     </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:38:37</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>ヒョロガリが増量しない言い訳
+・体質的に太れない
+・食べるのが苦手
+・太ったらモテない
+・食費が高い
+モテボディを目指していても、
+太りつつ筋肉を増やす期間は必要。
+今から始めれば、来年に良い思いが出来る。
+俺はこのマインドで去年14kg増やした。</t>
+        </is>
+      </c>
+      <c r="C2140" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2140" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2140" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2140" t="inlineStr">
+        <is>
+          <t>【ヒョロガリ向け】最短で「モテボディ」を獲得するための食事プログラム｜by元体重39kgのヒョロガリが解説。
+https://note.com/puregrinding1/n/na60936ff3ad1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add smartphone addiction time loss post (row 2141)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2140"/>
+  <dimension ref="A1:G2141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62999,6 +62999,45 @@
         </is>
       </c>
     </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:46:54</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>スマホ中毒者は、
+・1日3時間
+・1ヶ月で 90時間
+・1年で 1,095時間
+・10年で 10,950時間
+を失っています。
+中毒を治し、
+「モテ」「金」「筋トレ」「スキル」
+に時間を投じましょう。
+どんなに怠惰な人間でも3時間は減らせる。
+ニートで1日10時間のスクロールガイガイの僕でも出来ました。</t>
+        </is>
+      </c>
+      <c r="C2141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2141" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2141" t="inlineStr">
+        <is>
+          <t>【スマホ中毒者向け】デジタル・ドーパミン廃人だった私がスクリーンタイム10時間→1時間で人生を奪還した思考法
+https://note.com/puregrinding1/n/n75b3881b4678</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add porn addiction post (row 2142)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2141"/>
+  <dimension ref="A1:G2142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63038,6 +63038,42 @@
         </is>
       </c>
     </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:02:31</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>ポルノ中毒で射精障害になる人の特徴は
+・過激なものにシフトしている
+・脚ピン、握力MAX、床でやる
+・三人称視点のポルノを好む
+俺も童卒した頃に実感した。
+EDまではいかないが、寝バックで強い刺激を与えないとイケなかった。
+童貞は初セスクで恥をかかないためにも、
+気を付けた方がいい。</t>
+        </is>
+      </c>
+      <c r="C2142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2142" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2142" t="inlineStr">
+        <is>
+          <t>「爆速でモテる男磨きのやり方」非モテが恋愛の土台を築き上げる男磨きby元自閉症チー牛が解説
+https://note.com/puregrinding1/n/n4eabc4c9b556</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add convenience store 850yen post with image (row 2143)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2142"/>
+  <dimension ref="A1:G2143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63074,6 +63074,42 @@
         </is>
       </c>
     </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>2026-10-24 19:21:13</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>「コンビニ飯850円は高い」とか舐めんな。
+ヒョロガリと貧乏人は850円使って、
+スーパーで全卵40個買え。</t>
+        </is>
+      </c>
+      <c r="C2143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2143" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2143" t="inlineStr">
+        <is>
+          <t>【ヒョロガリ向け】最短で「モテボディ」を獲得するための食事プログラム｜by元体重39kgのヒョロガリが解説。
+https://note.com/puregrinding1/n/na60936ff3ad1</t>
+        </is>
+      </c>
+      <c r="G2143" t="inlineStr">
+        <is>
+          <t>images/convenience_store_850.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add motivation content post (row 2144, no image yet)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2143"/>
+  <dimension ref="A1:G2144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63110,6 +63110,37 @@
         </is>
       </c>
     </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>2026-10-24 19:23:55</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>人生がつまらなかったら、
+ギラギラしたコンテンツを見るといい。
+女、金、自由という「男のシンプルな欲望」を刺激してみてください。
+TikTok等で「wolfofwallstreetedit」「Billionaire motivation」と検索するとピッタリな動画が出てきます。</t>
+        </is>
+      </c>
+      <c r="C2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2144" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove motivation content post (row 2144)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2144"/>
+  <dimension ref="A1:G2143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63110,37 +63110,6 @@
         </is>
       </c>
     </row>
-    <row r="2144">
-      <c r="A2144" t="inlineStr">
-        <is>
-          <t>2026-10-24 19:23:55</t>
-        </is>
-      </c>
-      <c r="B2144" t="inlineStr">
-        <is>
-          <t>人生がつまらなかったら、
-ギラギラしたコンテンツを見るといい。
-女、金、自由という「男のシンプルな欲望」を刺激してみてください。
-TikTok等で「wolfofwallstreetedit」「Billionaire motivation」と検索するとピッタリな動画が出てきます。</t>
-        </is>
-      </c>
-      <c r="C2144" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2144" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2144" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="F2144" t="inlineStr">
-        <is>
-          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add chee-gyu and delayed gratification posts (rows 2144-2145)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2143"/>
+  <dimension ref="A1:G2145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63110,6 +63110,78 @@
         </is>
       </c>
     </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>2026-10-24 23:47:16</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>チー牛を卒業する男
+・自分から話しかける
+・断られても次に行く
+・遺伝的限界までベストを尽くす
+チー牛のままの奴
+・顔のせいにする
+・男磨き陰キャのまま
+・モテテクだけ集める
+容姿は大事。
+でも、分かれ目は自己完結に逃げないこと。
+自閉チー牛の私も男磨き陰キャやめて、対人関係と向き合ってから彼女ができました。</t>
+        </is>
+      </c>
+      <c r="C2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2144" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>「爆速でモテる男磨きのやり方」非モテが恋愛の土台を築き上げる男磨きby元自閉症チー牛が解説
+https://note.com/puregrinding1/n/n4eabc4c9b556</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>2026-10-24 23:47:16</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>弱者男性は「報酬を先送りにする能力」に欠けている。
+スマホ中毒しかり、貧困層にフードデリバリーの利用率が高いのも領ける。(確かイギリスのuberのデータ)
+今を犠牲にして、将来に報酬を先送りにする。
+これだけ覚えておくだけで、人生は変わる。
+スマホ廃人の私もそうでした。</t>
+        </is>
+      </c>
+      <c r="C2145" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2145" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2145" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2145" t="inlineStr">
+        <is>
+          <t>【スマホ中毒者向け】"デジタル・ドーパミン廃人"だった私がスクリーンタイム10時間→1時間で人生を奪還した思考法
+https://note.com/puregrinding1/n/n75b3881b4678</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add weak man reversal post (row 2146)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2145"/>
+  <dimension ref="A1:G2146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63182,6 +63182,39 @@
         </is>
       </c>
     </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>2026-10-25 20:30:01</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>弱男はスマホをやめて、運動習慣取り入れる。
+そして支出は最大限カットして、
+空き時間で出来る月5万のビジネスを作る。
+それをさらに自己投資して稼ぐ。
+そしたら、逆転への道が切り開ける。
+20代だったらモテ攻略も遅くはない。</t>
+        </is>
+      </c>
+      <c r="C2146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2146" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2146" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2146" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add habits and environment post (row 2147)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2146"/>
+  <dimension ref="A1:G2147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63215,6 +63215,44 @@
         </is>
       </c>
     </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>2026-10-27 10:54:15</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>成長している時は常にダサい。
+習慣化は「距離」が命。
+・徒歩で行けるジムを選ぶ
+・作業専用の書斎を作る
+・目標を壁紙にする
+逆に悪習慣は遠ざける。
+・スマホを別室に置く
+・アプリを遠ざけるor消す
+・衝動買い
+→クレカを財布から抜く
+環境を変えれば、習慣は勝手に変わる。</t>
+        </is>
+      </c>
+      <c r="C2147" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2147" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2147" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2147" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ugly growth phase post (row 2148)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2147"/>
+  <dimension ref="A1:G2148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63253,6 +63253,43 @@
         </is>
       </c>
     </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>2026-10-27 10:54:44</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>成長している時は常にダサい。
+・男磨き全般
+・童貞のキモアプローチ
+・ヒョロガリがジムに行く時
+ここで「冷笑対象になるならやめるわ」となる奴は
+メンタル的に向いていない。
+逆にダサいと思われても「だからなんや？」と
+なれる人はそのまま成長できる。
+まずダサい時期を乗り越えろ。</t>
+        </is>
+      </c>
+      <c r="C2148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2148" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2148" t="inlineStr">
+        <is>
+          <t>「爆速でモテる男磨きのやり方」非モテが恋愛の土台を築き上げる男磨きby元自閉症チー牛が解説
+https://note.com/puregrinding1/n/n4eabc4c9b556</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix dates for rows 2140-2148 to make them eligible for scheduling
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -62965,7 +62965,7 @@
     <row r="2140">
       <c r="A2140" t="inlineStr">
         <is>
-          <t>2026-10-22 18:38:37</t>
+          <t>2026-08-10 00:00:00</t>
         </is>
       </c>
       <c r="B2140" t="inlineStr">
@@ -63002,7 +63002,7 @@
     <row r="2141">
       <c r="A2141" t="inlineStr">
         <is>
-          <t>2026-10-22 18:46:54</t>
+          <t>2026-08-11 00:00:00</t>
         </is>
       </c>
       <c r="B2141" t="inlineStr">
@@ -63041,7 +63041,7 @@
     <row r="2142">
       <c r="A2142" t="inlineStr">
         <is>
-          <t>2026-10-22 20:02:31</t>
+          <t>2026-08-12 00:00:00</t>
         </is>
       </c>
       <c r="B2142" t="inlineStr">
@@ -63077,7 +63077,7 @@
     <row r="2143">
       <c r="A2143" t="inlineStr">
         <is>
-          <t>2026-10-24 19:21:13</t>
+          <t>2026-08-13 00:00:00</t>
         </is>
       </c>
       <c r="B2143" t="inlineStr">
@@ -63113,7 +63113,7 @@
     <row r="2144">
       <c r="A2144" t="inlineStr">
         <is>
-          <t>2026-10-24 23:47:16</t>
+          <t>2026-08-14 00:00:00</t>
         </is>
       </c>
       <c r="B2144" t="inlineStr">
@@ -63152,7 +63152,7 @@
     <row r="2145">
       <c r="A2145" t="inlineStr">
         <is>
-          <t>2026-10-24 23:47:16</t>
+          <t>2026-08-15 00:00:00</t>
         </is>
       </c>
       <c r="B2145" t="inlineStr">
@@ -63185,7 +63185,7 @@
     <row r="2146">
       <c r="A2146" t="inlineStr">
         <is>
-          <t>2026-10-25 20:30:01</t>
+          <t>2026-08-16 00:00:00</t>
         </is>
       </c>
       <c r="B2146" t="inlineStr">
@@ -63218,7 +63218,7 @@
     <row r="2147">
       <c r="A2147" t="inlineStr">
         <is>
-          <t>2026-10-27 10:54:15</t>
+          <t>2026-08-17 00:00:00</t>
         </is>
       </c>
       <c r="B2147" t="inlineStr">
@@ -63256,7 +63256,7 @@
     <row r="2148">
       <c r="A2148" t="inlineStr">
         <is>
-          <t>2026-10-27 10:54:44</t>
+          <t>2026-08-18 00:00:00</t>
         </is>
       </c>
       <c r="B2148" t="inlineStr">

</xml_diff>